<commit_message>
ppt & tableau update
</commit_message>
<xml_diff>
--- a/ssp_modeling/input_data/reference/morocco_ghg_scenarios.xlsx
+++ b/ssp_modeling/input_data/reference/morocco_ghg_scenarios.xlsx
@@ -5,28 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_morocco/ssp_modeling/input_data/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD068C8-CB12-3B4D-A897-FF10732408DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA206307-19C2-D047-963C-A948B8984102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-39640" yWindow="600" windowWidth="36200" windowHeight="24680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GHG Scenarios" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'GHG Scenarios'!$A$4</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'GHG Scenarios'!$A$5:$A$33</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'GHG Scenarios'!$B$4</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'GHG Scenarios'!$B$5:$B$33</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'GHG Scenarios'!$C$4</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'GHG Scenarios'!$C$5:$C$33</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'GHG Scenarios'!$D$4</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'GHG Scenarios'!$D$5:$D$33</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'GHG Scenarios'!$E$4</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'GHG Scenarios'!$E$5:$E$33</definedName>
-  </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -48,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>Morocco — National GHG Emissions: Reference (BAU) vs Net Zero (SNBC)</t>
   </si>
@@ -57,12 +45,6 @@
   </si>
   <si>
     <t>Year</t>
-  </si>
-  <si>
-    <t>Reference (MtCO2eq)</t>
-  </si>
-  <si>
-    <t>Net Zero (MtCO2eq)</t>
   </si>
   <si>
     <t>Note:</t>
@@ -74,7 +56,22 @@
     <t>LEDS</t>
   </si>
   <si>
-    <t>BAU</t>
+    <t>Pathway</t>
+  </si>
+  <si>
+    <t>Business as Usual</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net Zero </t>
+  </si>
+  <si>
+    <t>BAU - SSP</t>
+  </si>
+  <si>
+    <t>LEDS - SSP</t>
   </si>
 </sst>
 </file>
@@ -82,7 +79,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -186,8 +183,6 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -201,12 +196,14 @@
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -321,7 +318,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Reference (MtCO2eq)</c:v>
+                  <c:v>Reference</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -606,7 +603,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Net Zero (MtCO2eq)</c:v>
+                  <c:v>Net Zero </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -891,7 +888,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>BAU</c:v>
+                  <c:v>BAU - SSP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1038,94 +1035,94 @@
             <c:numRef>
               <c:f>'GHG Scenarios'!$D$5:$D$43</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.0</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="39"/>
                 <c:pt idx="0">
-                  <c:v>108.49615109154696</c:v>
+                  <c:v>108.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>109.9939405035454</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>112.58681054488552</c:v>
+                  <c:v>112.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>114.96640609240885</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>117.52042312318602</c:v>
+                  <c:v>117.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>120.08631864124736</c:v>
+                  <c:v>120.1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>122.6656140152928</c:v>
+                  <c:v>122.7</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>125.27658513368426</c:v>
+                  <c:v>125.3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>127.89904535966082</c:v>
+                  <c:v>127.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>130.53402639779492</c:v>
+                  <c:v>130.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>133.18291939371198</c:v>
+                  <c:v>133.19999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>135.84724118327981</c:v>
+                  <c:v>135.80000000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>138.52866199432543</c:v>
+                  <c:v>138.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>141.22910648274689</c:v>
+                  <c:v>141.19999999999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>143.95067894724733</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>146.69594235436296</c:v>
+                  <c:v>146.69999999999999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>149.46847192959163</c:v>
+                  <c:v>149.5</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>152.27287717331933</c:v>
+                  <c:v>152.30000000000001</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>155.11348944669896</c:v>
+                  <c:v>155.1</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>158.01790324222586</c:v>
+                  <c:v>158</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>160.99601413802696</c:v>
+                  <c:v>161</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>164.05505652483436</c:v>
+                  <c:v>164.1</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>167.19622329996861</c:v>
+                  <c:v>167.2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>170.42280904812816</c:v>
+                  <c:v>170.4</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>173.74996191238216</c:v>
+                  <c:v>173.7</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>177.17867095208862</c:v>
+                  <c:v>177.2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>180.66163907156604</c:v>
+                  <c:v>180.7</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>184.21071690382442</c:v>
+                  <c:v>184.2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>187.93653004971401</c:v>
+                  <c:v>187.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1146,7 +1143,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>LEDS</c:v>
+                  <c:v>LEDS - SSP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1293,94 +1290,94 @@
             <c:numRef>
               <c:f>'GHG Scenarios'!$E$5:$E$43</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.0</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="39"/>
                 <c:pt idx="0">
-                  <c:v>108.49610495153298</c:v>
+                  <c:v>108.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>108.63804919663119</c:v>
+                  <c:v>108.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>107.71620155624875</c:v>
+                  <c:v>108</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>106.20543175681527</c:v>
+                  <c:v>106.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>102.60423123335086</c:v>
+                  <c:v>103.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>98.953090248723285</c:v>
+                  <c:v>99.7</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>95.248294298315457</c:v>
+                  <c:v>96.1</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>91.450113013737962</c:v>
+                  <c:v>92.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>87.518161748388763</c:v>
+                  <c:v>88.7</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>83.391823984918332</c:v>
+                  <c:v>84.7</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>79.020269463020398</c:v>
+                  <c:v>80.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>74.394781914255418</c:v>
+                  <c:v>76.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>69.405722937272074</c:v>
+                  <c:v>71.3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>64.049231637861794</c:v>
+                  <c:v>66.2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>58.438113886973746</c:v>
+                  <c:v>60.9</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>52.786242738124407</c:v>
+                  <c:v>55.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>47.299840717352005</c:v>
+                  <c:v>50.3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>42.093734350897378</c:v>
+                  <c:v>45.3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>37.174020083046997</c:v>
+                  <c:v>40.6</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>32.502494674477532</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>28.026626480159504</c:v>
+                  <c:v>31.7</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>23.70373213599629</c:v>
+                  <c:v>27.5</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>19.508021565738126</c:v>
+                  <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>15.407498704278364</c:v>
+                  <c:v>19.5</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>11.37369705030571</c:v>
+                  <c:v>15.6</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>7.3778947627067959</c:v>
+                  <c:v>11.8</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>3.4059282906511603</c:v>
+                  <c:v>7.9</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-0.56622995897111394</c:v>
+                  <c:v>4.0999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-4.5766928565358747</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1473,6 +1470,55 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>MTCO2e</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-MX"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -2149,9 +2195,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>417285</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>9070</xdr:rowOff>
+      <xdr:colOff>517071</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2358,7 +2404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:AJ89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -2366,655 +2412,1341 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="3">
+        <v>105</v>
+      </c>
+      <c r="C5" s="3">
+        <v>103</v>
+      </c>
+      <c r="D5">
+        <v>108.5</v>
+      </c>
+      <c r="E5">
+        <v>108.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>2023</v>
+      </c>
+      <c r="B6" s="3">
+        <v>108</v>
+      </c>
+      <c r="C6" s="3">
+        <v>105</v>
+      </c>
+      <c r="D6">
+        <v>110</v>
+      </c>
+      <c r="E6">
+        <v>108.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="3">
+        <v>110</v>
+      </c>
+      <c r="C7" s="3">
+        <v>102</v>
+      </c>
+      <c r="D7">
+        <v>112.6</v>
+      </c>
+      <c r="E7">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B8" s="3">
+        <v>113</v>
+      </c>
+      <c r="C8" s="3">
+        <v>99</v>
+      </c>
+      <c r="D8">
+        <v>115</v>
+      </c>
+      <c r="E8">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="3">
+        <v>115</v>
+      </c>
+      <c r="C9" s="3">
+        <v>96</v>
+      </c>
+      <c r="D9">
+        <v>117.5</v>
+      </c>
+      <c r="E9">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>2027</v>
+      </c>
+      <c r="B10" s="3">
+        <v>117</v>
+      </c>
+      <c r="C10" s="3">
+        <v>95</v>
+      </c>
+      <c r="D10">
+        <v>120.1</v>
+      </c>
+      <c r="E10">
+        <v>99.7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>2028</v>
+      </c>
+      <c r="B11" s="3">
+        <v>122</v>
+      </c>
+      <c r="C11" s="3">
+        <v>94</v>
+      </c>
+      <c r="D11">
+        <v>122.7</v>
+      </c>
+      <c r="E11">
+        <v>96.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>2029</v>
+      </c>
+      <c r="B12" s="3">
+        <v>128</v>
+      </c>
+      <c r="C12" s="3">
+        <v>94</v>
+      </c>
+      <c r="D12">
+        <v>125.3</v>
+      </c>
+      <c r="E12">
+        <v>92.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>2030</v>
+      </c>
+      <c r="B13" s="3">
+        <v>132</v>
+      </c>
+      <c r="C13" s="3">
+        <v>95</v>
+      </c>
+      <c r="D13">
+        <v>127.9</v>
+      </c>
+      <c r="E13">
+        <v>88.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>2031</v>
+      </c>
+      <c r="B14" s="3">
+        <v>138</v>
+      </c>
+      <c r="C14" s="3">
+        <v>95</v>
+      </c>
+      <c r="D14">
+        <v>130.5</v>
+      </c>
+      <c r="E14">
+        <v>84.7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>2032</v>
+      </c>
+      <c r="B15" s="3">
+        <v>140</v>
+      </c>
+      <c r="C15" s="3">
+        <v>95</v>
+      </c>
+      <c r="D15">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="E15">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>2033</v>
+      </c>
+      <c r="B16" s="3">
+        <v>141</v>
+      </c>
+      <c r="C16" s="3">
+        <v>93</v>
+      </c>
+      <c r="D16">
+        <v>135.80000000000001</v>
+      </c>
+      <c r="E16">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>2034</v>
+      </c>
+      <c r="B17" s="3">
+        <v>142</v>
+      </c>
+      <c r="C17" s="3">
+        <v>90</v>
+      </c>
+      <c r="D17">
+        <v>138.5</v>
+      </c>
+      <c r="E17">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
+        <v>2035</v>
+      </c>
+      <c r="B18" s="3">
+        <v>145</v>
+      </c>
+      <c r="C18" s="3">
+        <v>82</v>
+      </c>
+      <c r="D18">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="E18">
+        <v>66.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>2036</v>
+      </c>
+      <c r="B19" s="3">
+        <v>148</v>
+      </c>
+      <c r="C19" s="3">
+        <v>75</v>
+      </c>
+      <c r="D19">
+        <v>144</v>
+      </c>
+      <c r="E19">
+        <v>60.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="2">
+        <v>2037</v>
+      </c>
+      <c r="B20" s="3">
+        <v>150</v>
+      </c>
+      <c r="C20" s="3">
+        <v>67</v>
+      </c>
+      <c r="D20">
+        <v>146.69999999999999</v>
+      </c>
+      <c r="E20">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>2038</v>
+      </c>
+      <c r="B21" s="3">
+        <v>152</v>
+      </c>
+      <c r="C21" s="3">
+        <v>60</v>
+      </c>
+      <c r="D21">
+        <v>149.5</v>
+      </c>
+      <c r="E21">
+        <v>50.3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>2039</v>
+      </c>
+      <c r="B22" s="3">
+        <v>154</v>
+      </c>
+      <c r="C22" s="3">
+        <v>50</v>
+      </c>
+      <c r="D22">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="E22">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>2040</v>
+      </c>
+      <c r="B23" s="3">
+        <v>158</v>
+      </c>
+      <c r="C23" s="3">
+        <v>42</v>
+      </c>
+      <c r="D23">
+        <v>155.1</v>
+      </c>
+      <c r="E23">
+        <v>40.6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>2041</v>
+      </c>
+      <c r="B24" s="3">
+        <v>161</v>
+      </c>
+      <c r="C24" s="3">
+        <v>35</v>
+      </c>
+      <c r="D24">
+        <v>158</v>
+      </c>
+      <c r="E24">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>2042</v>
+      </c>
+      <c r="B25" s="3">
+        <v>163</v>
+      </c>
+      <c r="C25" s="3">
+        <v>30</v>
+      </c>
+      <c r="D25">
+        <v>161</v>
+      </c>
+      <c r="E25">
+        <v>31.7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
+        <v>2043</v>
+      </c>
+      <c r="B26" s="3">
+        <v>165</v>
+      </c>
+      <c r="C26" s="3">
+        <v>27</v>
+      </c>
+      <c r="D26">
+        <v>164.1</v>
+      </c>
+      <c r="E26">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
+        <v>2044</v>
+      </c>
+      <c r="B27" s="3">
+        <v>167</v>
+      </c>
+      <c r="C27" s="3">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <v>167.2</v>
+      </c>
+      <c r="E27">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
+        <v>2045</v>
+      </c>
+      <c r="B28" s="3">
+        <v>167</v>
+      </c>
+      <c r="C28" s="3">
+        <v>22</v>
+      </c>
+      <c r="D28">
+        <v>170.4</v>
+      </c>
+      <c r="E28">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>2046</v>
+      </c>
+      <c r="B29" s="3">
+        <v>167</v>
+      </c>
+      <c r="C29" s="3">
+        <v>19</v>
+      </c>
+      <c r="D29">
+        <v>173.7</v>
+      </c>
+      <c r="E29">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="2">
+        <v>2047</v>
+      </c>
+      <c r="B30" s="3">
+        <v>168</v>
+      </c>
+      <c r="C30" s="3">
+        <v>17</v>
+      </c>
+      <c r="D30">
+        <v>177.2</v>
+      </c>
+      <c r="E30">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>2048</v>
+      </c>
+      <c r="B31" s="3">
+        <v>169</v>
+      </c>
+      <c r="C31" s="3">
+        <v>14</v>
+      </c>
+      <c r="D31">
+        <v>180.7</v>
+      </c>
+      <c r="E31">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>2049</v>
+      </c>
+      <c r="B32" s="3">
+        <v>170</v>
+      </c>
+      <c r="C32" s="3">
+        <v>12</v>
+      </c>
+      <c r="D32">
+        <v>184.2</v>
+      </c>
+      <c r="E32">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>2050</v>
+      </c>
+      <c r="B33" s="5">
+        <v>172</v>
+      </c>
+      <c r="C33" s="5">
+        <v>8</v>
+      </c>
+      <c r="D33">
+        <v>187.9</v>
+      </c>
+      <c r="E33">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>2051</v>
+      </c>
+      <c r="B34" s="3">
+        <v>175</v>
+      </c>
+      <c r="C34" s="3">
+        <v>5</v>
+      </c>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>2052</v>
+      </c>
+      <c r="B35" s="3">
+        <v>178</v>
+      </c>
+      <c r="C35" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>2053</v>
+      </c>
+      <c r="B36" s="3">
+        <v>182</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>2054</v>
+      </c>
+      <c r="B37" s="3">
+        <v>187</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2</v>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>2055</v>
+      </c>
+      <c r="B38" s="3">
+        <v>190</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
+        <v>2056</v>
+      </c>
+      <c r="B39" s="3">
+        <v>195</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>2057</v>
+      </c>
+      <c r="B40" s="3">
+        <v>200</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>2058</v>
+      </c>
+      <c r="B41" s="3">
+        <v>205</v>
+      </c>
+      <c r="C41" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>2059</v>
+      </c>
+      <c r="B42" s="3">
+        <v>209</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>2060</v>
+      </c>
+      <c r="B43" s="3">
+        <v>213</v>
+      </c>
+      <c r="C43" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="C45" s="9"/>
+    </row>
+    <row r="52" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C52" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52">
+        <v>2018</v>
+      </c>
+      <c r="E52">
+        <v>2019</v>
+      </c>
+      <c r="F52">
+        <v>2020</v>
+      </c>
+      <c r="G52">
+        <v>2021</v>
+      </c>
+      <c r="H52">
+        <v>2022</v>
+      </c>
+      <c r="I52">
+        <v>2023</v>
+      </c>
+      <c r="J52">
+        <v>2024</v>
+      </c>
+      <c r="K52">
+        <v>2025</v>
+      </c>
+      <c r="L52">
+        <v>2026</v>
+      </c>
+      <c r="M52">
+        <v>2027</v>
+      </c>
+      <c r="N52">
+        <v>2028</v>
+      </c>
+      <c r="O52">
+        <v>2029</v>
+      </c>
+      <c r="P52">
+        <v>2030</v>
+      </c>
+      <c r="Q52">
+        <v>2031</v>
+      </c>
+      <c r="R52">
+        <v>2032</v>
+      </c>
+      <c r="S52">
+        <v>2033</v>
+      </c>
+      <c r="T52">
+        <v>2034</v>
+      </c>
+      <c r="U52">
+        <v>2035</v>
+      </c>
+      <c r="V52">
+        <v>2036</v>
+      </c>
+      <c r="W52">
+        <v>2037</v>
+      </c>
+      <c r="X52">
+        <v>2038</v>
+      </c>
+      <c r="Y52">
+        <v>2039</v>
+      </c>
+      <c r="Z52">
+        <v>2040</v>
+      </c>
+      <c r="AA52">
+        <v>2041</v>
+      </c>
+      <c r="AB52">
+        <v>2042</v>
+      </c>
+      <c r="AC52">
+        <v>2043</v>
+      </c>
+      <c r="AD52">
+        <v>2044</v>
+      </c>
+      <c r="AE52">
+        <v>2045</v>
+      </c>
+      <c r="AF52">
+        <v>2046</v>
+      </c>
+      <c r="AG52">
+        <v>2047</v>
+      </c>
+      <c r="AH52">
+        <v>2048</v>
+      </c>
+      <c r="AI52">
+        <v>2049</v>
+      </c>
+      <c r="AJ52">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="53" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C53" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="4">
+      <c r="D53">
+        <v>98.5</v>
+      </c>
+      <c r="E53">
+        <v>105.5</v>
+      </c>
+      <c r="F53">
+        <v>103.2</v>
+      </c>
+      <c r="G53">
+        <v>108.4</v>
+      </c>
+      <c r="H53">
+        <v>108.5</v>
+      </c>
+      <c r="I53">
+        <v>110</v>
+      </c>
+      <c r="J53">
+        <v>112.6</v>
+      </c>
+      <c r="K53">
+        <v>115</v>
+      </c>
+      <c r="L53">
+        <v>117.5</v>
+      </c>
+      <c r="M53">
+        <v>120.1</v>
+      </c>
+      <c r="N53">
+        <v>122.7</v>
+      </c>
+      <c r="O53">
+        <v>125.3</v>
+      </c>
+      <c r="P53">
+        <v>127.9</v>
+      </c>
+      <c r="Q53">
+        <v>130.5</v>
+      </c>
+      <c r="R53">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="S53">
+        <v>135.80000000000001</v>
+      </c>
+      <c r="T53">
+        <v>138.5</v>
+      </c>
+      <c r="U53">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="V53">
+        <v>144</v>
+      </c>
+      <c r="W53">
+        <v>146.69999999999999</v>
+      </c>
+      <c r="X53">
+        <v>149.5</v>
+      </c>
+      <c r="Y53">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="Z53">
+        <v>155.1</v>
+      </c>
+      <c r="AA53">
+        <v>158</v>
+      </c>
+      <c r="AB53">
+        <v>161</v>
+      </c>
+      <c r="AC53">
+        <v>164.1</v>
+      </c>
+      <c r="AD53">
+        <v>167.2</v>
+      </c>
+      <c r="AE53">
+        <v>170.4</v>
+      </c>
+      <c r="AF53">
+        <v>173.7</v>
+      </c>
+      <c r="AG53">
+        <v>177.2</v>
+      </c>
+      <c r="AH53">
+        <v>180.7</v>
+      </c>
+      <c r="AI53">
+        <v>184.2</v>
+      </c>
+      <c r="AJ53">
+        <v>187.9</v>
+      </c>
+    </row>
+    <row r="54" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C54" t="s">
+        <v>5</v>
+      </c>
+      <c r="D54">
+        <v>98.5</v>
+      </c>
+      <c r="E54">
+        <v>105.5</v>
+      </c>
+      <c r="F54">
+        <v>103.2</v>
+      </c>
+      <c r="G54">
+        <v>108.4</v>
+      </c>
+      <c r="H54">
+        <v>108.5</v>
+      </c>
+      <c r="I54">
+        <v>108.8</v>
+      </c>
+      <c r="J54">
+        <v>108</v>
+      </c>
+      <c r="K54">
+        <v>106.6</v>
+      </c>
+      <c r="L54">
+        <v>103.2</v>
+      </c>
+      <c r="M54">
+        <v>99.7</v>
+      </c>
+      <c r="N54">
+        <v>96.1</v>
+      </c>
+      <c r="O54">
+        <v>92.5</v>
+      </c>
+      <c r="P54">
+        <v>88.7</v>
+      </c>
+      <c r="Q54">
+        <v>84.7</v>
+      </c>
+      <c r="R54">
+        <v>80.5</v>
+      </c>
+      <c r="S54">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="T54">
+        <v>71.3</v>
+      </c>
+      <c r="U54">
+        <v>66.2</v>
+      </c>
+      <c r="V54">
+        <v>60.9</v>
+      </c>
+      <c r="W54">
+        <v>55.5</v>
+      </c>
+      <c r="X54">
+        <v>50.3</v>
+      </c>
+      <c r="Y54">
+        <v>45.3</v>
+      </c>
+      <c r="Z54">
+        <v>40.6</v>
+      </c>
+      <c r="AA54">
+        <v>36</v>
+      </c>
+      <c r="AB54">
+        <v>31.7</v>
+      </c>
+      <c r="AC54">
+        <v>27.5</v>
+      </c>
+      <c r="AD54">
+        <v>23.5</v>
+      </c>
+      <c r="AE54">
+        <v>19.5</v>
+      </c>
+      <c r="AF54">
+        <v>15.6</v>
+      </c>
+      <c r="AG54">
+        <v>11.8</v>
+      </c>
+      <c r="AH54">
+        <v>7.9</v>
+      </c>
+      <c r="AI54">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ54">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="56" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" t="s">
+        <v>7</v>
+      </c>
+      <c r="E56" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C57">
+        <v>2018</v>
+      </c>
+      <c r="D57">
+        <v>98.5</v>
+      </c>
+      <c r="E57">
+        <v>98.5</v>
+      </c>
+    </row>
+    <row r="58" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C58">
+        <v>2019</v>
+      </c>
+      <c r="D58">
+        <v>105.5</v>
+      </c>
+      <c r="E58">
+        <v>105.5</v>
+      </c>
+    </row>
+    <row r="59" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C59">
+        <v>2020</v>
+      </c>
+      <c r="D59">
+        <v>103.2</v>
+      </c>
+      <c r="E59">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="60" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C60">
+        <v>2021</v>
+      </c>
+      <c r="D60">
+        <v>108.4</v>
+      </c>
+      <c r="E60">
+        <v>108.4</v>
+      </c>
+    </row>
+    <row r="61" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C61">
         <v>2022</v>
       </c>
-      <c r="B5" s="5">
-        <v>105</v>
-      </c>
-      <c r="C5" s="5">
-        <v>103</v>
-      </c>
-      <c r="D5" s="8">
-        <v>108.49615109154696</v>
-      </c>
-      <c r="E5" s="8">
-        <v>108.49610495153298</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
+      <c r="D61">
+        <v>108.5</v>
+      </c>
+      <c r="E61">
+        <v>108.5</v>
+      </c>
+    </row>
+    <row r="62" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C62">
         <v>2023</v>
       </c>
-      <c r="B6" s="5">
+      <c r="D62">
+        <v>110</v>
+      </c>
+      <c r="E62">
+        <v>108.8</v>
+      </c>
+    </row>
+    <row r="63" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C63">
+        <v>2024</v>
+      </c>
+      <c r="D63">
+        <v>112.6</v>
+      </c>
+      <c r="E63">
         <v>108</v>
       </c>
-      <c r="C6" s="5">
-        <v>105</v>
-      </c>
-      <c r="D6" s="8">
-        <v>109.9939405035454</v>
-      </c>
-      <c r="E6" s="8">
-        <v>108.63804919663119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>2024</v>
-      </c>
-      <c r="B7" s="5">
-        <v>110</v>
-      </c>
-      <c r="C7" s="5">
-        <v>102</v>
-      </c>
-      <c r="D7" s="8">
-        <v>112.58681054488552</v>
-      </c>
-      <c r="E7" s="8">
-        <v>107.71620155624875</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+    </row>
+    <row r="64" spans="3:36" x14ac:dyDescent="0.2">
+      <c r="C64">
         <v>2025</v>
       </c>
-      <c r="B8" s="5">
-        <v>113</v>
-      </c>
-      <c r="C8" s="5">
-        <v>99</v>
-      </c>
-      <c r="D8" s="8">
-        <v>114.96640609240885</v>
-      </c>
-      <c r="E8" s="8">
-        <v>106.20543175681527</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
+      <c r="D64">
+        <v>115</v>
+      </c>
+      <c r="E64">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="65" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C65">
         <v>2026</v>
       </c>
-      <c r="B9" s="5">
-        <v>115</v>
-      </c>
-      <c r="C9" s="5">
-        <v>96</v>
-      </c>
-      <c r="D9" s="8">
-        <v>117.52042312318602</v>
-      </c>
-      <c r="E9" s="8">
-        <v>102.60423123335086</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
+      <c r="D65">
+        <v>117.5</v>
+      </c>
+      <c r="E65">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="66" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C66">
         <v>2027</v>
       </c>
-      <c r="B10" s="5">
-        <v>117</v>
-      </c>
-      <c r="C10" s="5">
-        <v>95</v>
-      </c>
-      <c r="D10" s="8">
-        <v>120.08631864124736</v>
-      </c>
-      <c r="E10" s="8">
-        <v>98.953090248723285</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
+      <c r="D66">
+        <v>120.1</v>
+      </c>
+      <c r="E66">
+        <v>99.7</v>
+      </c>
+    </row>
+    <row r="67" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C67">
         <v>2028</v>
       </c>
-      <c r="B11" s="5">
-        <v>122</v>
-      </c>
-      <c r="C11" s="5">
-        <v>94</v>
-      </c>
-      <c r="D11" s="8">
-        <v>122.6656140152928</v>
-      </c>
-      <c r="E11" s="8">
-        <v>95.248294298315457</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="4">
+      <c r="D67">
+        <v>122.7</v>
+      </c>
+      <c r="E67">
+        <v>96.1</v>
+      </c>
+    </row>
+    <row r="68" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C68">
         <v>2029</v>
       </c>
-      <c r="B12" s="5">
-        <v>128</v>
-      </c>
-      <c r="C12" s="5">
-        <v>94</v>
-      </c>
-      <c r="D12" s="8">
-        <v>125.27658513368426</v>
-      </c>
-      <c r="E12" s="8">
-        <v>91.450113013737962</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="4">
+      <c r="D68">
+        <v>125.3</v>
+      </c>
+      <c r="E68">
+        <v>92.5</v>
+      </c>
+    </row>
+    <row r="69" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C69">
         <v>2030</v>
       </c>
-      <c r="B13" s="5">
-        <v>132</v>
-      </c>
-      <c r="C13" s="5">
-        <v>95</v>
-      </c>
-      <c r="D13" s="8">
-        <v>127.89904535966082</v>
-      </c>
-      <c r="E13" s="8">
-        <v>87.518161748388763</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
+      <c r="D69">
+        <v>127.9</v>
+      </c>
+      <c r="E69">
+        <v>88.7</v>
+      </c>
+    </row>
+    <row r="70" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C70">
         <v>2031</v>
       </c>
-      <c r="B14" s="5">
-        <v>138</v>
-      </c>
-      <c r="C14" s="5">
-        <v>95</v>
-      </c>
-      <c r="D14" s="8">
-        <v>130.53402639779492</v>
-      </c>
-      <c r="E14" s="8">
-        <v>83.391823984918332</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="4">
+      <c r="D70">
+        <v>130.5</v>
+      </c>
+      <c r="E70">
+        <v>84.7</v>
+      </c>
+    </row>
+    <row r="71" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C71">
         <v>2032</v>
       </c>
-      <c r="B15" s="5">
-        <v>140</v>
-      </c>
-      <c r="C15" s="5">
-        <v>95</v>
-      </c>
-      <c r="D15" s="8">
-        <v>133.18291939371198</v>
-      </c>
-      <c r="E15" s="8">
-        <v>79.020269463020398</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
+      <c r="D71">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="E71">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="72" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C72">
         <v>2033</v>
       </c>
-      <c r="B16" s="5">
-        <v>141</v>
-      </c>
-      <c r="C16" s="5">
-        <v>93</v>
-      </c>
-      <c r="D16" s="8">
-        <v>135.84724118327981</v>
-      </c>
-      <c r="E16" s="8">
-        <v>74.394781914255418</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
+      <c r="D72">
+        <v>135.80000000000001</v>
+      </c>
+      <c r="E72">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="73" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C73">
         <v>2034</v>
       </c>
-      <c r="B17" s="5">
-        <v>142</v>
-      </c>
-      <c r="C17" s="5">
-        <v>90</v>
-      </c>
-      <c r="D17" s="8">
-        <v>138.52866199432543</v>
-      </c>
-      <c r="E17" s="8">
-        <v>69.405722937272074</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
+      <c r="D73">
+        <v>138.5</v>
+      </c>
+      <c r="E73">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="74" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C74">
         <v>2035</v>
       </c>
-      <c r="B18" s="5">
-        <v>145</v>
-      </c>
-      <c r="C18" s="5">
-        <v>82</v>
-      </c>
-      <c r="D18" s="8">
-        <v>141.22910648274689</v>
-      </c>
-      <c r="E18" s="8">
-        <v>64.049231637861794</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="4">
+      <c r="D74">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="E74">
+        <v>66.2</v>
+      </c>
+    </row>
+    <row r="75" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C75">
         <v>2036</v>
       </c>
-      <c r="B19" s="5">
-        <v>148</v>
-      </c>
-      <c r="C19" s="5">
-        <v>75</v>
-      </c>
-      <c r="D19" s="8">
-        <v>143.95067894724733</v>
-      </c>
-      <c r="E19" s="8">
-        <v>58.438113886973746</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="4">
+      <c r="D75">
+        <v>144</v>
+      </c>
+      <c r="E75">
+        <v>60.9</v>
+      </c>
+    </row>
+    <row r="76" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C76">
         <v>2037</v>
       </c>
-      <c r="B20" s="5">
-        <v>150</v>
-      </c>
-      <c r="C20" s="5">
-        <v>67</v>
-      </c>
-      <c r="D20" s="8">
-        <v>146.69594235436296</v>
-      </c>
-      <c r="E20" s="8">
-        <v>52.786242738124407</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="4">
+      <c r="D76">
+        <v>146.69999999999999</v>
+      </c>
+      <c r="E76">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="77" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C77">
         <v>2038</v>
       </c>
-      <c r="B21" s="5">
-        <v>152</v>
-      </c>
-      <c r="C21" s="5">
-        <v>60</v>
-      </c>
-      <c r="D21" s="8">
-        <v>149.46847192959163</v>
-      </c>
-      <c r="E21" s="8">
-        <v>47.299840717352005</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="4">
+      <c r="D77">
+        <v>149.5</v>
+      </c>
+      <c r="E77">
+        <v>50.3</v>
+      </c>
+    </row>
+    <row r="78" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C78">
         <v>2039</v>
       </c>
-      <c r="B22" s="5">
-        <v>154</v>
-      </c>
-      <c r="C22" s="5">
-        <v>50</v>
-      </c>
-      <c r="D22" s="8">
-        <v>152.27287717331933</v>
-      </c>
-      <c r="E22" s="8">
-        <v>42.093734350897378</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="4">
+      <c r="D78">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="E78">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="79" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C79">
         <v>2040</v>
       </c>
-      <c r="B23" s="5">
+      <c r="D79">
+        <v>155.1</v>
+      </c>
+      <c r="E79">
+        <v>40.6</v>
+      </c>
+    </row>
+    <row r="80" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C80">
+        <v>2041</v>
+      </c>
+      <c r="D80">
         <v>158</v>
       </c>
-      <c r="C23" s="5">
-        <v>42</v>
-      </c>
-      <c r="D23" s="8">
-        <v>155.11348944669896</v>
-      </c>
-      <c r="E23" s="8">
-        <v>37.174020083046997</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="4">
-        <v>2041</v>
-      </c>
-      <c r="B24" s="5">
+      <c r="E80">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="81" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C81">
+        <v>2042</v>
+      </c>
+      <c r="D81">
         <v>161</v>
       </c>
-      <c r="C24" s="5">
-        <v>35</v>
-      </c>
-      <c r="D24" s="8">
-        <v>158.01790324222586</v>
-      </c>
-      <c r="E24" s="8">
-        <v>32.502494674477532</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="4">
-        <v>2042</v>
-      </c>
-      <c r="B25" s="5">
-        <v>163</v>
-      </c>
-      <c r="C25" s="5">
-        <v>30</v>
-      </c>
-      <c r="D25" s="8">
-        <v>160.99601413802696</v>
-      </c>
-      <c r="E25" s="8">
-        <v>28.026626480159504</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="4">
+      <c r="E81">
+        <v>31.7</v>
+      </c>
+    </row>
+    <row r="82" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C82">
         <v>2043</v>
       </c>
-      <c r="B26" s="5">
-        <v>165</v>
-      </c>
-      <c r="C26" s="5">
-        <v>27</v>
-      </c>
-      <c r="D26" s="8">
-        <v>164.05505652483436</v>
-      </c>
-      <c r="E26" s="8">
-        <v>23.70373213599629</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="4">
+      <c r="D82">
+        <v>164.1</v>
+      </c>
+      <c r="E82">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="83" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C83">
         <v>2044</v>
       </c>
-      <c r="B27" s="5">
-        <v>167</v>
-      </c>
-      <c r="C27" s="5">
-        <v>25</v>
-      </c>
-      <c r="D27" s="8">
-        <v>167.19622329996861</v>
-      </c>
-      <c r="E27" s="8">
-        <v>19.508021565738126</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="4">
+      <c r="D83">
+        <v>167.2</v>
+      </c>
+      <c r="E83">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="84" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C84">
         <v>2045</v>
       </c>
-      <c r="B28" s="5">
-        <v>167</v>
-      </c>
-      <c r="C28" s="5">
-        <v>22</v>
-      </c>
-      <c r="D28" s="8">
-        <v>170.42280904812816</v>
-      </c>
-      <c r="E28" s="8">
-        <v>15.407498704278364</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="4">
+      <c r="D84">
+        <v>170.4</v>
+      </c>
+      <c r="E84">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="85" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C85">
         <v>2046</v>
       </c>
-      <c r="B29" s="5">
-        <v>167</v>
-      </c>
-      <c r="C29" s="5">
-        <v>19</v>
-      </c>
-      <c r="D29" s="8">
-        <v>173.74996191238216</v>
-      </c>
-      <c r="E29" s="8">
-        <v>11.37369705030571</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="4">
+      <c r="D85">
+        <v>173.7</v>
+      </c>
+      <c r="E85">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="86" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C86">
         <v>2047</v>
       </c>
-      <c r="B30" s="5">
-        <v>168</v>
-      </c>
-      <c r="C30" s="5">
-        <v>17</v>
-      </c>
-      <c r="D30" s="8">
-        <v>177.17867095208862</v>
-      </c>
-      <c r="E30" s="8">
-        <v>7.3778947627067959</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="4">
+      <c r="D86">
+        <v>177.2</v>
+      </c>
+      <c r="E86">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="87" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C87">
         <v>2048</v>
       </c>
-      <c r="B31" s="5">
-        <v>169</v>
-      </c>
-      <c r="C31" s="5">
-        <v>14</v>
-      </c>
-      <c r="D31" s="8">
-        <v>180.66163907156604</v>
-      </c>
-      <c r="E31" s="8">
-        <v>3.4059282906511603</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="4">
+      <c r="D87">
+        <v>180.7</v>
+      </c>
+      <c r="E87">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="88" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C88">
         <v>2049</v>
       </c>
-      <c r="B32" s="5">
-        <v>170</v>
-      </c>
-      <c r="C32" s="5">
-        <v>12</v>
-      </c>
-      <c r="D32" s="8">
-        <v>184.21071690382442</v>
-      </c>
-      <c r="E32" s="8">
-        <v>-0.56622995897111394</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="4">
+      <c r="D88">
+        <v>184.2</v>
+      </c>
+      <c r="E88">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="89" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C89">
         <v>2050</v>
       </c>
-      <c r="B33" s="7">
-        <v>172</v>
-      </c>
-      <c r="C33" s="7">
-        <v>8</v>
-      </c>
-      <c r="D33" s="8">
-        <v>187.93653004971401</v>
-      </c>
-      <c r="E33" s="8">
-        <v>-4.5766928565358747</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="4">
-        <v>2051</v>
-      </c>
-      <c r="B34" s="5">
-        <v>175</v>
-      </c>
-      <c r="C34" s="5">
-        <v>5</v>
-      </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="4">
-        <v>2052</v>
-      </c>
-      <c r="B35" s="5">
-        <v>178</v>
-      </c>
-      <c r="C35" s="5">
-        <v>3</v>
-      </c>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="4">
-        <v>2053</v>
-      </c>
-      <c r="B36" s="5">
-        <v>182</v>
-      </c>
-      <c r="C36" s="5">
-        <v>2</v>
-      </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="4">
-        <v>2054</v>
-      </c>
-      <c r="B37" s="5">
-        <v>187</v>
-      </c>
-      <c r="C37" s="5">
-        <v>2</v>
-      </c>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="4">
-        <v>2055</v>
-      </c>
-      <c r="B38" s="5">
-        <v>190</v>
-      </c>
-      <c r="C38" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="4">
-        <v>2056</v>
-      </c>
-      <c r="B39" s="5">
-        <v>195</v>
-      </c>
-      <c r="C39" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="4">
-        <v>2057</v>
-      </c>
-      <c r="B40" s="5">
-        <v>200</v>
-      </c>
-      <c r="C40" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="4">
-        <v>2058</v>
-      </c>
-      <c r="B41" s="5">
-        <v>205</v>
-      </c>
-      <c r="C41" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="4">
-        <v>2059</v>
-      </c>
-      <c r="B42" s="5">
-        <v>209</v>
-      </c>
-      <c r="C42" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="4">
-        <v>2060</v>
-      </c>
-      <c r="B43" s="5">
-        <v>213</v>
-      </c>
-      <c r="C43" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="1"/>
+      <c r="D89">
+        <v>187.9</v>
+      </c>
+      <c r="E89">
+        <v>0.2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>